<commit_message>
Zet 65 al bevestigde oude bronnen door naar de kolom Bron (geverifieerd)
Bij de controle van de 496 bestaande bronnen landde de uitkomst alleen in
"Status oude bron". Daardoor telden 65 vragen waarvan de pagina het antwoord
gewoon noemt mee als onbevestigd.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vragen/vragen_review_compleet.xlsx
+++ b/vragen/vragen_review_compleet.xlsx
@@ -959,6 +959,21 @@
         </is>
       </c>
       <c r="N5" s="4" t="n"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>https://www.who.int/news-room/spotlight/history-of-vaccination/history-of-smallpox-vaccination</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S5" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -1125,6 +1140,21 @@
           <t>geen bron</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/King_penguin</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S8" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -1227,6 +1257,21 @@
           <t>geen bron</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>https://www.ifaw.org/international/journal/fastest-whales-dolphins-ocean</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S10" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -1281,6 +1326,21 @@
         </is>
       </c>
       <c r="N11" s="4" t="n"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Crab</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S11" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -1388,6 +1448,21 @@
           <t>geen bron</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>https://www.coca-cola.com/ng/en/about-us/faq/how-much-sugar-is-in-cocacola-original-taste</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S13" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -2063,6 +2138,21 @@
         </is>
       </c>
       <c r="N25" s="4" t="n"/>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>https://www.esbnyc.com/about/facts-figures</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S25" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -2789,6 +2879,21 @@
         </is>
       </c>
       <c r="N39" s="4" t="n"/>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>https://plimoth.org/learn/just-kids/homework-help/mayflower</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S39" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -4583,6 +4688,21 @@
         </is>
       </c>
       <c r="N74" s="4" t="n"/>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>https://www.rsc.org/periodic-table/element/79/gold</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S74" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -6270,6 +6390,21 @@
         </is>
       </c>
       <c r="N107" s="4" t="n"/>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/conditions/blood-groups/</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S107" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -6814,6 +6949,21 @@
         </is>
       </c>
       <c r="N118" s="4" t="n"/>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>https://www.mouthhealthy.org/all-topics-a-z/eruption-charts</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S118" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -7005,6 +7155,21 @@
         </is>
       </c>
       <c r="N122" s="4" t="n"/>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>https://www.nidcd.nih.gov/health/taste-disorders</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S122" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -7330,6 +7495,21 @@
         </is>
       </c>
       <c r="N128" s="4" t="n"/>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>https://www.genome.gov/human-genome-project/Completion-FAQ</t>
+        </is>
+      </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S128" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -8421,6 +8601,21 @@
         </is>
       </c>
       <c r="N150" s="4" t="n"/>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>https://animals.sandiegozoo.org/animals/camel</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S150" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -8465,6 +8660,21 @@
         </is>
       </c>
       <c r="N151" s="4" t="n"/>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>https://animals.sandiegozoo.org/animals/camel</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S151" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -9614,6 +9824,21 @@
         </is>
       </c>
       <c r="N173" s="4" t="n"/>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>https://www.bceao.int/en/content/west-african-cfa-franc</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R173" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S173" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -9826,6 +10051,21 @@
         </is>
       </c>
       <c r="N177" s="4" t="n"/>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>https://www.g7italy.it/en/about-g7/</t>
+        </is>
+      </c>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S177" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -12059,6 +12299,21 @@
         </is>
       </c>
       <c r="N219" s="4" t="n"/>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>https://www.berlin.de/en/attractions-and-sights/3560266-3104050-brandenburg-gate.en.html</t>
+        </is>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R219" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S219" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -12304,6 +12559,21 @@
         </is>
       </c>
       <c r="N224" s="4" t="n"/>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>https://asi.nic.in/taj-mahal/</t>
+        </is>
+      </c>
+      <c r="P224" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R224" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S224" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -20076,6 +20346,21 @@
         </is>
       </c>
       <c r="N375" s="4" t="n"/>
+      <c r="O375" t="inlineStr">
+        <is>
+          <t>https://www.ipcc.ch/report/ar6/wg1/chapter/chapter-5/</t>
+        </is>
+      </c>
+      <c r="P375" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R375" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S375" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -20331,6 +20616,21 @@
         </is>
       </c>
       <c r="N380" s="4" t="n"/>
+      <c r="O380" t="inlineStr">
+        <is>
+          <t>https://www.usgs.gov/special-topics/water-science-school/science/where-earths-water</t>
+        </is>
+      </c>
+      <c r="P380" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R380" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S380" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -21320,6 +21620,21 @@
         </is>
       </c>
       <c r="N399" s="4" t="n"/>
+      <c r="O399" t="inlineStr">
+        <is>
+          <t>https://www.yamaha.com/en/musical_instrument_guide/piano/structure/</t>
+        </is>
+      </c>
+      <c r="P399" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R399" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S399" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -22760,6 +23075,21 @@
         </is>
       </c>
       <c r="N426" s="4" t="n"/>
+      <c r="O426" t="inlineStr">
+        <is>
+          <t>https://www.conseil-constitutionnel.fr/en/declaration-of-human-and-civic-rights-of-26-august-1789</t>
+        </is>
+      </c>
+      <c r="P426" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R426" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S426" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -22902,6 +23232,21 @@
         </is>
       </c>
       <c r="N429" s="4" t="n"/>
+      <c r="O429" t="inlineStr">
+        <is>
+          <t>https://www.nato.int/cps/en/natohq/topics_52044.htm</t>
+        </is>
+      </c>
+      <c r="P429" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R429" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S429" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -23117,6 +23462,21 @@
         </is>
       </c>
       <c r="N433" s="4" t="n"/>
+      <c r="O433" t="inlineStr">
+        <is>
+          <t>https://www.nato.int/cps/en/natolive/topics_52044.htm</t>
+        </is>
+      </c>
+      <c r="P433" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R433" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S433" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -24684,6 +25044,21 @@
         </is>
       </c>
       <c r="N463" s="4" t="n"/>
+      <c r="O463" t="inlineStr">
+        <is>
+          <t>https://openstax.org/books/chemistry-2e/pages/7-2-covalent-bonding</t>
+        </is>
+      </c>
+      <c r="P463" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R463" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S463" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -24728,6 +25103,21 @@
         </is>
       </c>
       <c r="N464" s="4" t="n"/>
+      <c r="O464" t="inlineStr">
+        <is>
+          <t>https://openstax.org/books/chemistry-2e/pages/2-3-atomic-structure-and-symbolism</t>
+        </is>
+      </c>
+      <c r="P464" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R464" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S464" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -24860,6 +25250,21 @@
         </is>
       </c>
       <c r="N467" s="4" t="n"/>
+      <c r="O467" t="inlineStr">
+        <is>
+          <t>https://pubchem.ncbi.nlm.nih.gov/compound/Carbon-dioxide</t>
+        </is>
+      </c>
+      <c r="P467" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R467" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S467" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -25100,6 +25505,21 @@
         </is>
       </c>
       <c r="N472" s="4" t="n"/>
+      <c r="O472" t="inlineStr">
+        <is>
+          <t>https://iupac.org/what-we-do/periodic-table-of-elements/</t>
+        </is>
+      </c>
+      <c r="P472" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R472" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S472" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -25144,6 +25564,21 @@
         </is>
       </c>
       <c r="N473" s="4" t="n"/>
+      <c r="O473" t="inlineStr">
+        <is>
+          <t>https://www.ecfr.gov/current/title-21/chapter-I/subchapter-B/part-169</t>
+        </is>
+      </c>
+      <c r="P473" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R473" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S473" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -25188,6 +25623,21 @@
         </is>
       </c>
       <c r="N474" s="4" t="n"/>
+      <c r="O474" t="inlineStr">
+        <is>
+          <t>https://www.rsc.org/periodic-table/element/92/uranium</t>
+        </is>
+      </c>
+      <c r="P474" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R474" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S474" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -25232,6 +25682,21 @@
         </is>
       </c>
       <c r="N475" s="4" t="n"/>
+      <c r="O475" t="inlineStr">
+        <is>
+          <t>https://www.rsc.org/periodic-table/element/74/tungsten</t>
+        </is>
+      </c>
+      <c r="P475" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R475" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S475" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -25330,6 +25795,21 @@
         </is>
       </c>
       <c r="N477" s="4" t="n"/>
+      <c r="O477" t="inlineStr">
+        <is>
+          <t>https://www.usgs.gov/special-topics/water-science-school/science/ph-and-water</t>
+        </is>
+      </c>
+      <c r="P477" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R477" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S477" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -26067,6 +26547,21 @@
         </is>
       </c>
       <c r="N491" s="4" t="n"/>
+      <c r="O491" t="inlineStr">
+        <is>
+          <t>https://handbook.fide.com/chapter/E012023</t>
+        </is>
+      </c>
+      <c r="P491" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R491" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S491" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -26530,6 +27025,21 @@
         </is>
       </c>
       <c r="N500" s="4" t="n"/>
+      <c r="O500" t="inlineStr">
+        <is>
+          <t>https://operations.nfl.com/the-rules/nfl-rulebook/</t>
+        </is>
+      </c>
+      <c r="P500" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R500" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S500" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -26716,6 +27226,21 @@
         </is>
       </c>
       <c r="N504" s="4" t="n"/>
+      <c r="O504" t="inlineStr">
+        <is>
+          <t>https://www.theifab.com/laws/latest/the-players/</t>
+        </is>
+      </c>
+      <c r="P504" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R504" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S504" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -27015,6 +27540,21 @@
         </is>
       </c>
       <c r="N510" s="4" t="n"/>
+      <c r="O510" t="inlineStr">
+        <is>
+          <t>https://science.nasa.gov/jupiter/facts/</t>
+        </is>
+      </c>
+      <c r="P510" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R510" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S510" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -27059,6 +27599,21 @@
         </is>
       </c>
       <c r="N511" s="4" t="n"/>
+      <c r="O511" t="inlineStr">
+        <is>
+          <t>https://science.nasa.gov/venus/venus-facts/</t>
+        </is>
+      </c>
+      <c r="P511" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R511" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S511" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -27103,6 +27658,21 @@
         </is>
       </c>
       <c r="N512" s="4" t="n"/>
+      <c r="O512" t="inlineStr">
+        <is>
+          <t>https://science.nasa.gov/neptune/facts/</t>
+        </is>
+      </c>
+      <c r="P512" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R512" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S512" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -28345,6 +28915,21 @@
         </is>
       </c>
       <c r="N536" s="4" t="n"/>
+      <c r="O536" t="inlineStr">
+        <is>
+          <t>https://science.nasa.gov/moon/facts/</t>
+        </is>
+      </c>
+      <c r="P536" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R536" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S536" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -30329,6 +30914,21 @@
         </is>
       </c>
       <c r="N574" s="4" t="n"/>
+      <c r="O574" t="inlineStr">
+        <is>
+          <t>https://tfl.gov.uk/corporate/about-tfl/what-we-do/london-underground</t>
+        </is>
+      </c>
+      <c r="P574" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R574" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S574" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -30373,9 +30973,24 @@
         </is>
       </c>
       <c r="N575" s="4" t="n"/>
+      <c r="O575" t="inlineStr">
+        <is>
+          <t>https://www.airbus.com/en/products-services/commercial-aircraft/passenger-aircraft/a380</t>
+        </is>
+      </c>
+      <c r="P575" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
       <c r="Q575" t="inlineStr">
         <is>
           <t>Wikidata: klopt</t>
+        </is>
+      </c>
+      <c r="R575" t="inlineStr">
+        <is>
+          <t>hoog</t>
         </is>
       </c>
       <c r="S575" t="inlineStr">
@@ -32097,6 +32712,21 @@
         </is>
       </c>
       <c r="N609" s="4" t="n"/>
+      <c r="O609" t="inlineStr">
+        <is>
+          <t>https://www.ncbi.nlm.nih.gov/books/NBK470353/</t>
+        </is>
+      </c>
+      <c r="P609" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R609" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S609" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -32141,6 +32771,21 @@
         </is>
       </c>
       <c r="N610" s="4" t="n"/>
+      <c r="O610" t="inlineStr">
+        <is>
+          <t>https://www.usgs.gov/special-topics/water-science-school/science/water-you-water-and-human-body</t>
+        </is>
+      </c>
+      <c r="P610" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R610" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S610" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -33631,6 +34276,21 @@
         </is>
       </c>
       <c r="N640" s="4" t="n"/>
+      <c r="O640" t="inlineStr">
+        <is>
+          <t>https://nationalzoo.si.edu/animals/aldabra-tortoise</t>
+        </is>
+      </c>
+      <c r="P640" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R640" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S640" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -34986,6 +35646,21 @@
         </is>
       </c>
       <c r="N665" s="4" t="n"/>
+      <c r="O665" t="inlineStr">
+        <is>
+          <t>https://flybase.org/</t>
+        </is>
+      </c>
+      <c r="P665" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R665" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S665" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -35133,6 +35808,21 @@
         </is>
       </c>
       <c r="N668" s="4" t="n"/>
+      <c r="O668" t="inlineStr">
+        <is>
+          <t>https://www.fisheries.noaa.gov/species/american-lobster</t>
+        </is>
+      </c>
+      <c r="P668" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R668" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S668" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -39583,6 +40273,21 @@
         </is>
       </c>
       <c r="N752" s="4" t="n"/>
+      <c r="O752" t="inlineStr">
+        <is>
+          <t>https://www.alpconv.org/en/home/</t>
+        </is>
+      </c>
+      <c r="P752" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R752" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S752" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -44508,6 +45213,21 @@
           <t>geen EN-vertaling</t>
         </is>
       </c>
+      <c r="O843" t="inlineStr">
+        <is>
+          <t>https://education.nationalgeographic.org/resource/equator/</t>
+        </is>
+      </c>
+      <c r="P843" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R843" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S843" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -55216,6 +55936,21 @@
         </is>
       </c>
       <c r="N1044" s="4" t="n"/>
+      <c r="O1044" t="inlineStr">
+        <is>
+          <t>https://www.fao.org/aquastat/en/overview/methodology/water-use</t>
+        </is>
+      </c>
+      <c r="P1044" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1044" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1044" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -64456,6 +65191,21 @@
         </is>
       </c>
       <c r="N1217" s="4" t="n"/>
+      <c r="O1217" t="inlineStr">
+        <is>
+          <t>https://www.un.org/en/about-us/history-of-the-un</t>
+        </is>
+      </c>
+      <c r="P1217" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1217" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1217" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -67256,6 +68006,21 @@
         </is>
       </c>
       <c r="N1270" s="4" t="n"/>
+      <c r="O1270" t="inlineStr">
+        <is>
+          <t>https://openstax.org/books/chemistry-2e/pages/2-3-atomic-structure-and-symbolism</t>
+        </is>
+      </c>
+      <c r="P1270" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1270" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1270" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -67359,6 +68124,21 @@
         </is>
       </c>
       <c r="N1272" s="4" t="n"/>
+      <c r="O1272" t="inlineStr">
+        <is>
+          <t>https://openstax.org/books/chemistry-2e/pages/7-2-covalent-bonding</t>
+        </is>
+      </c>
+      <c r="P1272" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1272" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1272" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -68199,6 +68979,21 @@
         </is>
       </c>
       <c r="N1288" s="4" t="n"/>
+      <c r="O1288" t="inlineStr">
+        <is>
+          <t>https://handbook.fide.com/chapter/E012023</t>
+        </is>
+      </c>
+      <c r="P1288" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1288" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1288" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -68792,6 +69587,21 @@
         </is>
       </c>
       <c r="N1299" s="4" t="n"/>
+      <c r="O1299" t="inlineStr">
+        <is>
+          <t>https://www.randa.org/en/rog/the-rules-of-golf</t>
+        </is>
+      </c>
+      <c r="P1299" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1299" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1299" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -68880,6 +69690,21 @@
         </is>
       </c>
       <c r="N1301" s="4" t="n"/>
+      <c r="O1301" t="inlineStr">
+        <is>
+          <t>https://www.randa.org/en/rog/the-rules-of-golf</t>
+        </is>
+      </c>
+      <c r="P1301" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1301" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1301" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -70272,6 +71097,21 @@
         </is>
       </c>
       <c r="N1327" s="4" t="n"/>
+      <c r="O1327" t="inlineStr">
+        <is>
+          <t>https://www.theifab.com/laws/latest/the-field-of-play/</t>
+        </is>
+      </c>
+      <c r="P1327" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1327" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1327" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -70472,6 +71312,21 @@
         </is>
       </c>
       <c r="N1331" s="4" t="n"/>
+      <c r="O1331" t="inlineStr">
+        <is>
+          <t>https://www.theifab.com/laws/latest/the-field-of-play/</t>
+        </is>
+      </c>
+      <c r="P1331" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1331" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1331" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -70727,6 +71582,21 @@
         </is>
       </c>
       <c r="N1336" s="4" t="n"/>
+      <c r="O1336" t="inlineStr">
+        <is>
+          <t>https://operations.nfl.com/the-rules/nfl-rulebook/</t>
+        </is>
+      </c>
+      <c r="P1336" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1336" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1336" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -72664,6 +73534,21 @@
         </is>
       </c>
       <c r="N1374" s="4" t="n"/>
+      <c r="O1374" t="inlineStr">
+        <is>
+          <t>https://science.nasa.gov/solar-system/planets/</t>
+        </is>
+      </c>
+      <c r="P1374" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1374" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1374" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -73333,6 +74218,21 @@
         </is>
       </c>
       <c r="N1387" s="4" t="n"/>
+      <c r="O1387" t="inlineStr">
+        <is>
+          <t>https://www.nasa.gov/mission/apollo-11/</t>
+        </is>
+      </c>
+      <c r="P1387" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1387" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1387" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -73677,6 +74577,21 @@
         </is>
       </c>
       <c r="N1394" s="4" t="n"/>
+      <c r="O1394" t="inlineStr">
+        <is>
+          <t>https://science.nasa.gov/sun/facts/</t>
+        </is>
+      </c>
+      <c r="P1394" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1394" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1394" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -74314,6 +75229,21 @@
           <t>geen EN-vertaling</t>
         </is>
       </c>
+      <c r="O1406" t="inlineStr">
+        <is>
+          <t>https://physics.nist.gov/cuu/Units/binary.html</t>
+        </is>
+      </c>
+      <c r="P1406" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1406" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1406" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -74358,6 +75288,21 @@
         </is>
       </c>
       <c r="N1407" s="4" t="n"/>
+      <c r="O1407" t="inlineStr">
+        <is>
+          <t>https://physics.nist.gov/cuu/Units/binary.html</t>
+        </is>
+      </c>
+      <c r="P1407" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1407" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1407" t="inlineStr">
         <is>
           <t>bevestigd</t>
@@ -75344,6 +76289,21 @@
         </is>
       </c>
       <c r="N1426" s="4" t="n"/>
+      <c r="O1426" t="inlineStr">
+        <is>
+          <t>https://www.ibm.com/history/floppy-disk</t>
+        </is>
+      </c>
+      <c r="P1426" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1426" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1426" t="inlineStr">
         <is>
           <t>getal gezien op de pagina</t>
@@ -76933,6 +77893,21 @@
         </is>
       </c>
       <c r="N1457" s="4" t="n"/>
+      <c r="O1457" t="inlineStr">
+        <is>
+          <t>https://mathworld.wolfram.com/Divisor.html</t>
+        </is>
+      </c>
+      <c r="P1457" t="inlineStr">
+        <is>
+          <t>Bestaande bron opgehaald; het antwoord staat op de pagina.</t>
+        </is>
+      </c>
+      <c r="R1457" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
       <c r="S1457" t="inlineStr">
         <is>
           <t>bevestigd</t>

</xml_diff>